<commit_message>
feat: deliver premium end-to-end Document AI course
</commit_message>
<xml_diff>
--- a/sample_outputs/receipt_result.xlsx
+++ b/sample_outputs/receipt_result.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="검토_요약" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="품목" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="원문" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="원문_근거" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,14 +425,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,7 +461,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>review_status</t>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>reviewer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>reviewed_at</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>change_reason</t>
         </is>
       </c>
     </row>
@@ -485,9 +503,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>사람 확인 완료</t>
-        </is>
-      </c>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>교육용 검수자</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,9 +537,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>사람 확인 완료</t>
-        </is>
-      </c>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>교육용 검수자</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -522,8 +554,10 @@
           <t>total_amount</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>5000</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
       </c>
       <c r="C4" t="n">
         <v>5000</v>
@@ -533,9 +567,16 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>사람 확인 완료</t>
-        </is>
-      </c>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>교육용 검수자</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -666,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -681,17 +722,101 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>mock</t>
+          <t>synthetic_fixture_rule_extraction</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>fixture_type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>input_file</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>input_sha256</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>engine_version</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>target_technology</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>reviewer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>ocr_text</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>{'store_name': {'raw_value': '샘플문구점', 'line': 1}, 'date': {'raw_value': '거래일자: 2026-07-27', 'line': 2}, 'total_amount': {'raw_value': '합계: 5,000원', 'line': 5}}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>